<commit_message>
Working on contert csv to json
</commit_message>
<xml_diff>
--- a/forms_data/Nutrição e práticas saudáveis(1-144).xlsx
+++ b/forms_data/Nutrição e práticas saudáveis(1-144).xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Claudio\Desktop\Projeto de EDF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-20.04\home\tuna\Projeto de EDF\forms_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3631" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3631" uniqueCount="150">
   <si>
     <t>ID</t>
   </si>
@@ -326,9 +326,6 @@
     <t>KickBoxing</t>
   </si>
   <si>
-    <t>Kickboxe</t>
-  </si>
-  <si>
     <t xml:space="preserve">Basquetebol </t>
   </si>
   <si>
@@ -345,9 +342,6 @@
   </si>
   <si>
     <t>Corrida</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kickboxing </t>
   </si>
   <si>
     <t>Hóquei em patins</t>
@@ -368,9 +362,6 @@
     <t xml:space="preserve">Hóquei em patins </t>
   </si>
   <si>
-    <t>KickBoxe</t>
-  </si>
-  <si>
     <t xml:space="preserve">Exercicios em casa </t>
   </si>
   <si>
@@ -381,9 +372,6 @@
   </si>
   <si>
     <t>Física;Psicologia B;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kickboxing/Muay-Thai </t>
   </si>
   <si>
     <t>Psicologia B;Geografia C;</t>
@@ -470,9 +458,6 @@
     <t xml:space="preserve">Futsal </t>
   </si>
   <si>
-    <t>Btt</t>
-  </si>
-  <si>
     <t xml:space="preserve">dança </t>
   </si>
   <si>
@@ -483,6 +468,12 @@
   </si>
   <si>
     <t>Dança, Pilates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KickBoxing/Muay Thai </t>
+  </si>
+  <si>
+    <t>BTT</t>
   </si>
 </sst>
 </file>
@@ -529,12 +520,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3969,7 +3961,7 @@
         <v>42</v>
       </c>
       <c r="V29" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="W29" s="3" t="s">
         <v>86</v>
@@ -4174,7 +4166,7 @@
         <v>42</v>
       </c>
       <c r="V31" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="W31" s="3" t="s">
         <v>67</v>
@@ -4280,7 +4272,7 @@
         <v>42</v>
       </c>
       <c r="V32" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="W32" s="3" t="s">
         <v>67</v>
@@ -4346,7 +4338,7 @@
         <v>69</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>83</v>
@@ -4453,7 +4445,7 @@
         <v>98</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I34" s="2">
         <v>185</v>
@@ -4687,7 +4679,7 @@
         <v>45</v>
       </c>
       <c r="S36" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="T36" s="3" t="s">
         <v>84</v>
@@ -4696,7 +4688,7 @@
         <v>42</v>
       </c>
       <c r="V36" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="W36" s="3" t="s">
         <v>67</v>
@@ -4901,7 +4893,7 @@
         <v>42</v>
       </c>
       <c r="V38" s="3" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="W38" s="3" t="s">
         <v>86</v>
@@ -5012,7 +5004,7 @@
         <v>42</v>
       </c>
       <c r="V39" s="3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="W39" s="3" t="s">
         <v>67</v>
@@ -5314,7 +5306,7 @@
         <v>42</v>
       </c>
       <c r="V42" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="W42" s="3" t="s">
         <v>67</v>
@@ -5479,7 +5471,7 @@
         <v>69</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H44" s="3" t="s">
         <v>60</v>
@@ -5524,7 +5516,7 @@
         <v>42</v>
       </c>
       <c r="V44" s="3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="W44" s="3" t="s">
         <v>67</v>
@@ -5585,7 +5577,7 @@
         <v>69</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H45" s="3" t="s">
         <v>62</v>
@@ -5729,7 +5721,7 @@
         <v>42</v>
       </c>
       <c r="V46" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="W46" s="3" t="s">
         <v>67</v>
@@ -5939,7 +5931,7 @@
         <v>42</v>
       </c>
       <c r="V48" s="3" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="W48" s="3" t="s">
         <v>86</v>
@@ -6048,7 +6040,7 @@
         <v>42</v>
       </c>
       <c r="V49" s="3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="W49" s="3" t="s">
         <v>86</v>
@@ -6205,7 +6197,7 @@
       </c>
       <c r="E51" s="3"/>
       <c r="F51" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G51" s="3" t="s">
         <v>61</v>
@@ -6307,10 +6299,10 @@
         <v>69</v>
       </c>
       <c r="G52" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="H52" s="3" t="s">
         <v>103</v>
-      </c>
-      <c r="H52" s="3" t="s">
-        <v>104</v>
       </c>
       <c r="I52" s="2">
         <v>181</v>
@@ -6352,7 +6344,7 @@
         <v>42</v>
       </c>
       <c r="V52" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="W52" s="3" t="s">
         <v>67</v>
@@ -6458,7 +6450,7 @@
         <v>42</v>
       </c>
       <c r="V53" s="3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="W53" s="3" t="s">
         <v>86</v>
@@ -6727,7 +6719,7 @@
         <v>69</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H56" s="3" t="s">
         <v>40</v>
@@ -6772,7 +6764,7 @@
         <v>42</v>
       </c>
       <c r="V56" s="3" t="s">
-        <v>119</v>
+        <v>148</v>
       </c>
       <c r="W56" s="3" t="s">
         <v>86</v>
@@ -6835,7 +6827,7 @@
       </c>
       <c r="E57" s="3"/>
       <c r="F57" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G57" s="3" t="s">
         <v>61</v>
@@ -6934,10 +6926,10 @@
       </c>
       <c r="E58" s="3"/>
       <c r="F58" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="G58" s="3" t="s">
         <v>116</v>
-      </c>
-      <c r="G58" s="3" t="s">
-        <v>120</v>
       </c>
       <c r="H58" s="3" t="s">
         <v>83</v>
@@ -7034,7 +7026,7 @@
         <v>69</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H59" s="3" t="s">
         <v>83</v>
@@ -7191,7 +7183,7 @@
         <v>6</v>
       </c>
       <c r="AA60" s="3" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="AB60" s="3" t="s">
         <v>46</v>
@@ -7287,7 +7279,7 @@
         <v>42</v>
       </c>
       <c r="V61" s="3" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="W61" s="3" t="s">
         <v>67</v>
@@ -7393,7 +7385,7 @@
         <v>42</v>
       </c>
       <c r="V62" s="3" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="W62" s="3" t="s">
         <v>67</v>
@@ -7860,7 +7852,7 @@
         <v>69</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H67" s="3" t="s">
         <v>92</v>
@@ -7905,7 +7897,7 @@
         <v>42</v>
       </c>
       <c r="V67" s="3" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="W67" s="3" t="s">
         <v>86</v>
@@ -7971,7 +7963,7 @@
         <v>69</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H68" s="3" t="s">
         <v>93</v>
@@ -8016,7 +8008,7 @@
         <v>42</v>
       </c>
       <c r="V68" s="3" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="W68" s="3" t="s">
         <v>86</v>
@@ -8077,7 +8069,7 @@
         <v>38</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="H69" s="3" t="s">
         <v>62</v>
@@ -8176,7 +8168,7 @@
         <v>38</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="H70" s="3" t="s">
         <v>62</v>
@@ -8316,7 +8308,7 @@
         <v>42</v>
       </c>
       <c r="V71" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="W71" s="3" t="s">
         <v>67</v>
@@ -8377,7 +8369,7 @@
         <v>69</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H72" s="3" t="s">
         <v>62</v>
@@ -8481,7 +8473,7 @@
         <v>69</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H73" s="3" t="s">
         <v>92</v>
@@ -8689,7 +8681,7 @@
         <v>38</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="H75" s="3" t="s">
         <v>60</v>
@@ -8734,7 +8726,7 @@
         <v>42</v>
       </c>
       <c r="V75" s="3" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="W75" s="3" t="s">
         <v>67</v>
@@ -8795,7 +8787,7 @@
         <v>38</v>
       </c>
       <c r="G76" s="3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="H76" s="3" t="s">
         <v>62</v>
@@ -8899,7 +8891,7 @@
         <v>38</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="H77" s="3" t="s">
         <v>83</v>
@@ -8998,7 +8990,7 @@
         <v>38</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="H78" s="3" t="s">
         <v>62</v>
@@ -9097,10 +9089,10 @@
         <v>38</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I79" s="3">
         <v>160</v>
@@ -9196,7 +9188,7 @@
         <v>38</v>
       </c>
       <c r="G80" s="3" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="H80" s="3" t="s">
         <v>83</v>
@@ -9394,7 +9386,7 @@
         <v>38</v>
       </c>
       <c r="G82" s="3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="H82" s="3" t="s">
         <v>60</v>
@@ -9493,7 +9485,7 @@
         <v>38</v>
       </c>
       <c r="G83" s="3" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="H83" s="3" t="s">
         <v>53</v>
@@ -9590,7 +9582,7 @@
         <v>38</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="H84" s="3" t="s">
         <v>93</v>
@@ -9635,7 +9627,7 @@
         <v>42</v>
       </c>
       <c r="V84" s="3" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="W84" s="3" t="s">
         <v>67</v>
@@ -9696,7 +9688,7 @@
         <v>38</v>
       </c>
       <c r="G85" s="3" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="H85" s="3" t="s">
         <v>83</v>
@@ -9795,7 +9787,7 @@
         <v>69</v>
       </c>
       <c r="G86" s="3" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="H86" s="3" t="s">
         <v>60</v>
@@ -9840,7 +9832,7 @@
         <v>42</v>
       </c>
       <c r="V86" s="3" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="W86" s="3" t="s">
         <v>86</v>
@@ -10000,7 +9992,7 @@
         <v>38</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="H88" s="3" t="s">
         <v>83</v>
@@ -10099,7 +10091,7 @@
         <v>38</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="H89" s="3" t="s">
         <v>60</v>
@@ -10294,10 +10286,10 @@
       </c>
       <c r="E91" s="3"/>
       <c r="F91" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G91" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="H91" s="3" t="s">
         <v>88</v>
@@ -10394,7 +10386,7 @@
         <v>38</v>
       </c>
       <c r="G92" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="H92" s="3" t="s">
         <v>60</v>
@@ -10741,7 +10733,7 @@
         <v>42</v>
       </c>
       <c r="V95" s="3" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="W95" s="3" t="s">
         <v>67</v>
@@ -10807,10 +10799,10 @@
         <v>38</v>
       </c>
       <c r="G96" s="3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="H96" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I96" s="2">
         <v>165</v>
@@ -11055,7 +11047,7 @@
         <v>42</v>
       </c>
       <c r="V98" s="3" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="W98" s="3" t="s">
         <v>86</v>
@@ -11166,7 +11158,7 @@
         <v>42</v>
       </c>
       <c r="V99" s="3" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="W99" s="3" t="s">
         <v>67</v>
@@ -11230,7 +11222,7 @@
         <v>65</v>
       </c>
       <c r="H100" s="3" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I100" s="2">
         <v>156</v>
@@ -11326,7 +11318,7 @@
         <v>69</v>
       </c>
       <c r="G101" s="3" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="H101" s="3" t="s">
         <v>62</v>
@@ -11477,7 +11469,7 @@
         <v>42</v>
       </c>
       <c r="V102" s="3" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="W102" s="3" t="s">
         <v>86</v>
@@ -11583,7 +11575,7 @@
         <v>42</v>
       </c>
       <c r="V103" s="3" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="W103" s="3" t="s">
         <v>86</v>
@@ -12088,7 +12080,7 @@
         <v>42</v>
       </c>
       <c r="V108" s="3" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="W108" s="3" t="s">
         <v>67</v>
@@ -12194,7 +12186,7 @@
         <v>42</v>
       </c>
       <c r="V109" s="3" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="W109" s="3" t="s">
         <v>67</v>
@@ -12399,7 +12391,7 @@
         <v>42</v>
       </c>
       <c r="V111" s="3" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="W111" s="3" t="s">
         <v>67</v>
@@ -12460,7 +12452,7 @@
         <v>69</v>
       </c>
       <c r="G112" s="3" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="H112" s="3" t="s">
         <v>62</v>
@@ -12505,7 +12497,7 @@
         <v>42</v>
       </c>
       <c r="V112" s="3" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="W112" s="3" t="s">
         <v>67</v>
@@ -12566,7 +12558,7 @@
         <v>38</v>
       </c>
       <c r="G113" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="H113" s="3" t="s">
         <v>88</v>
@@ -12665,7 +12657,7 @@
         <v>38</v>
       </c>
       <c r="G114" s="3" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="H114" s="3" t="s">
         <v>88</v>
@@ -12809,7 +12801,7 @@
         <v>42</v>
       </c>
       <c r="V115" s="3" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="W115" s="3" t="s">
         <v>67</v>
@@ -12873,7 +12865,7 @@
         <v>61</v>
       </c>
       <c r="H116" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I116" s="3">
         <v>178</v>
@@ -13220,7 +13212,7 @@
         <v>42</v>
       </c>
       <c r="V119" s="3" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="W119" s="3" t="s">
         <v>86</v>
@@ -13326,7 +13318,7 @@
         <v>42</v>
       </c>
       <c r="V120" s="3" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="W120" s="3" t="s">
         <v>86</v>
@@ -13341,7 +13333,7 @@
         <v>5</v>
       </c>
       <c r="AA120" s="3" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="AB120" s="3" t="s">
         <v>46</v>
@@ -13392,7 +13384,7 @@
         <v>69</v>
       </c>
       <c r="G121" s="3" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="H121" s="3" t="s">
         <v>62</v>
@@ -13696,13 +13688,13 @@
       </c>
       <c r="E124" s="3"/>
       <c r="F124" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G124" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="H124" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I124" s="2">
         <v>180</v>
@@ -14048,7 +14040,7 @@
         <v>42</v>
       </c>
       <c r="V127" s="3" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="W127" s="3" t="s">
         <v>67</v>
@@ -14154,7 +14146,7 @@
         <v>42</v>
       </c>
       <c r="V128" s="3" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="W128" s="3" t="s">
         <v>67</v>
@@ -14314,7 +14306,7 @@
       </c>
       <c r="E130" s="3"/>
       <c r="F130" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G130" s="3" t="s">
         <v>61</v>
@@ -14413,7 +14405,7 @@
       </c>
       <c r="E131" s="3"/>
       <c r="F131" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G131" s="3" t="s">
         <v>61</v>
@@ -14469,7 +14461,7 @@
         <v>6</v>
       </c>
       <c r="AA131" s="3" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="AB131" s="3" t="s">
         <v>46</v>
@@ -14517,10 +14509,10 @@
       </c>
       <c r="E132" s="3"/>
       <c r="F132" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="G132" s="3" t="s">
         <v>116</v>
-      </c>
-      <c r="G132" s="3" t="s">
-        <v>120</v>
       </c>
       <c r="H132" s="3" t="s">
         <v>40</v>
@@ -14623,7 +14615,7 @@
       </c>
       <c r="E133" s="3"/>
       <c r="F133" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G133" s="3" t="s">
         <v>61</v>
@@ -14671,7 +14663,7 @@
         <v>42</v>
       </c>
       <c r="V133" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="W133" s="3" t="s">
         <v>67</v>
@@ -14734,7 +14726,7 @@
       </c>
       <c r="E134" s="3"/>
       <c r="F134" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G134" s="3" t="s">
         <v>61</v>
@@ -14781,8 +14773,8 @@
       <c r="U134" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="V134" s="3" t="s">
-        <v>149</v>
+      <c r="V134" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="W134" s="3" t="s">
         <v>67</v>
@@ -14840,7 +14832,7 @@
       </c>
       <c r="E135" s="3"/>
       <c r="F135" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G135" s="3" t="s">
         <v>61</v>
@@ -14937,7 +14929,7 @@
       </c>
       <c r="E136" s="3"/>
       <c r="F136" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G136" s="3" t="s">
         <v>61</v>
@@ -15036,7 +15028,7 @@
       </c>
       <c r="E137" s="3"/>
       <c r="F137" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G137" s="3" t="s">
         <v>61</v>
@@ -15140,7 +15132,7 @@
       </c>
       <c r="E138" s="3"/>
       <c r="F138" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G138" s="3" t="s">
         <v>61</v>
@@ -15239,7 +15231,7 @@
       </c>
       <c r="E139" s="3"/>
       <c r="F139" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G139" s="3" t="s">
         <v>61</v>
@@ -15343,10 +15335,10 @@
       </c>
       <c r="E140" s="3"/>
       <c r="F140" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="G140" s="3" t="s">
         <v>116</v>
-      </c>
-      <c r="G140" s="3" t="s">
-        <v>120</v>
       </c>
       <c r="H140" s="3" t="s">
         <v>93</v>
@@ -15447,7 +15439,7 @@
       </c>
       <c r="E141" s="3"/>
       <c r="F141" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G141" s="3" t="s">
         <v>61</v>
@@ -15503,7 +15495,7 @@
         <v>6</v>
       </c>
       <c r="AA141" s="3" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="AB141" s="3" t="s">
         <v>46</v>
@@ -15551,7 +15543,7 @@
       </c>
       <c r="E142" s="3"/>
       <c r="F142" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G142" s="3" t="s">
         <v>61</v>
@@ -15599,7 +15591,7 @@
         <v>42</v>
       </c>
       <c r="V142" s="3" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="W142" s="3" t="s">
         <v>86</v>
@@ -15662,10 +15654,10 @@
       </c>
       <c r="E143" s="3"/>
       <c r="F143" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G143" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="H143" s="3" t="s">
         <v>60</v>
@@ -15768,10 +15760,10 @@
       </c>
       <c r="E144" s="3"/>
       <c r="F144" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G144" s="3" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="H144" s="3" t="s">
         <v>83</v>
@@ -15816,7 +15808,7 @@
         <v>42</v>
       </c>
       <c r="V144" s="3" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="W144" s="3" t="s">
         <v>67</v>
@@ -15874,10 +15866,10 @@
       </c>
       <c r="E145" s="3"/>
       <c r="F145" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="G145" s="3" t="s">
         <v>116</v>
-      </c>
-      <c r="G145" s="3" t="s">
-        <v>120</v>
       </c>
       <c r="H145" s="3" t="s">
         <v>83</v>

</xml_diff>

<commit_message>
Update Nutrição e práticas saudáveis(1-144).xlsx
</commit_message>
<xml_diff>
--- a/forms_data/Nutrição e práticas saudáveis(1-144).xlsx
+++ b/forms_data/Nutrição e práticas saudáveis(1-144).xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-20.04\home\tuna\Projeto de EDF\forms_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mestre.LAPTOP-GPBR\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D8F1D94-7FD1-4545-9A52-738E0D4C53D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7905"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nutrição e práticas saudáveis(1" sheetId="1" r:id="rId1"/>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3631" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3629" uniqueCount="139">
   <si>
     <t>ID</t>
   </si>
@@ -225,9 +226,6 @@
     <t>Psicologia B;Inglês;</t>
   </si>
   <si>
-    <t>Tenis</t>
-  </si>
-  <si>
     <t>Coletivo</t>
   </si>
   <si>
@@ -267,9 +265,6 @@
     <t>6-10</t>
   </si>
   <si>
-    <t xml:space="preserve">Dança </t>
-  </si>
-  <si>
     <t>Artes</t>
   </si>
   <si>
@@ -292,9 +287,6 @@
   </si>
   <si>
     <t>70-75kg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Futebol </t>
   </si>
   <si>
     <t>leve 1-3 dias por semana</t>
@@ -327,12 +319,6 @@
     <t>KickBoxing</t>
   </si>
   <si>
-    <t xml:space="preserve">Basquetebol </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Padel e Dança </t>
-  </si>
-  <si>
     <t>Física;Química;</t>
   </si>
   <si>
@@ -345,31 +331,13 @@
     <t>Corrida</t>
   </si>
   <si>
-    <t>Hóquei em patins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Costumo jogar futebol e andar de bicicleta </t>
-  </si>
-  <si>
     <t>Psicologia B;Biologia;</t>
-  </si>
-  <si>
-    <t>andebol e futsal</t>
   </si>
   <si>
     <t>Inglês;Física;</t>
   </si>
   <si>
-    <t xml:space="preserve">Hóquei em patins </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exercicios em casa </t>
-  </si>
-  <si>
     <t>Economia</t>
-  </si>
-  <si>
-    <t>Piscina</t>
   </si>
   <si>
     <t>Física;Psicologia B;</t>
@@ -381,28 +349,10 @@
     <t>&gt;2h</t>
   </si>
   <si>
-    <t xml:space="preserve">Natação </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Karaté </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crossfit </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muay Thai </t>
-  </si>
-  <si>
     <t>Inglês;Espanhol;</t>
   </si>
   <si>
-    <t xml:space="preserve">Bombos </t>
-  </si>
-  <si>
     <t>Geografia C;Espanhol;</t>
-  </si>
-  <si>
-    <t>corrida/caminhada</t>
   </si>
   <si>
     <t>40-45kg</t>
@@ -414,9 +364,6 @@
     <t>Inglês;História A;</t>
   </si>
   <si>
-    <t xml:space="preserve">Pólo Aquático </t>
-  </si>
-  <si>
     <t>Biologia;Física;</t>
   </si>
   <si>
@@ -426,43 +373,16 @@
     <t>Sociologia;Psicologia B;</t>
   </si>
   <si>
-    <t xml:space="preserve">Voleibol </t>
-  </si>
-  <si>
     <t>Ciclismo</t>
-  </si>
-  <si>
-    <t>Basketball</t>
   </si>
   <si>
     <t>Inglês;Biologia;</t>
   </si>
   <si>
-    <t>Basquetebol, Ténis de Campo e Ténis de Mesa</t>
-  </si>
-  <si>
-    <t>Polo aquático</t>
-  </si>
-  <si>
     <t>Pilates</t>
   </si>
   <si>
-    <t>hiphop</t>
-  </si>
-  <si>
     <t>Dança</t>
-  </si>
-  <si>
-    <t xml:space="preserve">corrida </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Futsal </t>
-  </si>
-  <si>
-    <t xml:space="preserve">dança </t>
-  </si>
-  <si>
-    <t>Ginásio</t>
   </si>
   <si>
     <t>Geografia C;Psicologia B;</t>
@@ -471,16 +391,64 @@
     <t>Dança, Pilates</t>
   </si>
   <si>
-    <t xml:space="preserve">KickBoxing/Muay Thai </t>
+    <t>Basquetebol</t>
   </si>
   <si>
-    <t>BTT</t>
+    <t>Padel Dança</t>
+  </si>
+  <si>
+    <t>Futebol Bicicleta</t>
+  </si>
+  <si>
+    <t>Ténis</t>
+  </si>
+  <si>
+    <t>Andebol Futsal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exercícios_em_casa </t>
+  </si>
+  <si>
+    <t>Hóquei_em_Patins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KickBoxing Muay Thai </t>
+  </si>
+  <si>
+    <t>Karaté</t>
+  </si>
+  <si>
+    <t>Crossfit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóquei_em_Patins </t>
+  </si>
+  <si>
+    <t>Muay_Thai</t>
+  </si>
+  <si>
+    <t>Bombos</t>
+  </si>
+  <si>
+    <t>Corrida Caminhada</t>
+  </si>
+  <si>
+    <t>Voleibol</t>
+  </si>
+  <si>
+    <t>Basquetebol Ténis Ténis_de_Mesa</t>
+  </si>
+  <si>
+    <t>Polo_Aquático</t>
+  </si>
+  <si>
+    <t>HipHop</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d/yy\ h:mm:ss"/>
   </numFmts>
@@ -658,46 +626,46 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:AK145" totalsRowShown="0">
-  <autoFilter ref="A1:AK145"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:AK145" totalsRowShown="0">
+  <autoFilter ref="A1:AK145" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="37">
-    <tableColumn id="1" name="ID" dataDxfId="36"/>
-    <tableColumn id="2" name="Start time" dataDxfId="35"/>
-    <tableColumn id="3" name="Completion time" dataDxfId="34"/>
-    <tableColumn id="4" name="Email" dataDxfId="33"/>
-    <tableColumn id="5" name="Name" dataDxfId="32"/>
-    <tableColumn id="6" name="Em qual curso te encontras?" dataDxfId="31"/>
-    <tableColumn id="7" name="Quais especificas frequentas?" dataDxfId="30"/>
-    <tableColumn id="8" name="Seleciona o intervalo que melhor enquadra o teu peso." dataDxfId="29"/>
-    <tableColumn id="9" name="Qual a tua altura em centímetros?" dataDxfId="28"/>
-    <tableColumn id="10" name="Sexo (biológico)." dataDxfId="27"/>
-    <tableColumn id="11" name="Quantas refeições fazes diariamente?" dataDxfId="26"/>
-    <tableColumn id="12" name="Costumas tomar o pequeno almoço?" dataDxfId="25"/>
-    <tableColumn id="13" name="Sabendo que o pequeno almoço é a refeição mais importante do dia, consideras o teu pequeno almoço saudável e adequado?" dataDxfId="24"/>
-    <tableColumn id="14" name="A tua alimentação diária respeita as porções na roda dos alimentos?" dataDxfId="23"/>
-    <tableColumn id="15" name="Quantas peças de fruta comes diariamente?" dataDxfId="22"/>
-    <tableColumn id="16" name="E quantas porções (aproximadamente a palma da mão) de legumes comes diariamente?" dataDxfId="21"/>
-    <tableColumn id="17" name="Sabes o consumo calórico diário recomendado para ti?" dataDxfId="20"/>
-    <tableColumn id="18" name="Consultas algum nutricionista?" dataDxfId="19"/>
-    <tableColumn id="19" name="Relativamente à tua alimentação tens alguma restrição?" dataDxfId="18"/>
-    <tableColumn id="20" name="Quantas vezes consomes &quot;fast food&quot; mensalmente?" dataDxfId="17"/>
-    <tableColumn id="21" name="Praticas alguma atividade física fora da escola? (Excepto ginásio)" dataDxfId="16"/>
-    <tableColumn id="22" name="Qual atividade praticas?" dataDxfId="15"/>
-    <tableColumn id="23" name="É uma atividade coletiva ou individual?" dataDxfId="14"/>
-    <tableColumn id="24" name="Quantas vezes praticas essa atividade semanalmente?" dataDxfId="13"/>
-    <tableColumn id="25" name="Frequentas o ginásio?" dataDxfId="12"/>
-    <tableColumn id="26" name="Quantos dias por semana vais ao ginásio?" dataDxfId="11"/>
-    <tableColumn id="27" name="Qual a duração média dos teus treinos? (ginásio)" dataDxfId="10"/>
-    <tableColumn id="28" name="Tiveste alguma lesão grave associada ao desporto, nos últimos 2 anos? (ex: fraturas, roturas, etc...)" dataDxfId="9"/>
-    <tableColumn id="29" name="No geral o teu exercício físico é..." dataDxfId="8"/>
-    <tableColumn id="30" name="Quantas horas costumas dormir, por dia, em média, durante a semana?" dataDxfId="7"/>
-    <tableColumn id="31" name="Quantas horas costumas dormir, por dia, em média, durante o fim de semana?" dataDxfId="6"/>
-    <tableColumn id="32" name="Costumas assistir algum tipo de ecrã até 30min antes de te deitares?" dataDxfId="5"/>
-    <tableColumn id="33" name="Costumas adormecer enquanto assistes conteúdos digital? (TV, Youtube, Netflix, TikTok, etc...)" dataDxfId="4"/>
-    <tableColumn id="34" name="Costumas comer antes de te deitares?" dataDxfId="3"/>
-    <tableColumn id="35" name="Costumas praticar atividades intensivas perto da hora de dormir?" dataDxfId="2"/>
-    <tableColumn id="36" name="Costumas tirar sestas durante o dia?" dataDxfId="1"/>
-    <tableColumn id="37" name="Costumas deitar-te sempre por volta da mesma hora?" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Start time" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Completion time" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Name" dataDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Em qual curso te encontras?" dataDxfId="31"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Quais especificas frequentas?" dataDxfId="30"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Seleciona o intervalo que melhor enquadra o teu peso." dataDxfId="29"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Qual a tua altura em centímetros?" dataDxfId="28"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Sexo (biológico)." dataDxfId="27"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Quantas refeições fazes diariamente?" dataDxfId="26"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Costumas tomar o pequeno almoço?" dataDxfId="25"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Sabendo que o pequeno almoço é a refeição mais importante do dia, consideras o teu pequeno almoço saudável e adequado?" dataDxfId="24"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="A tua alimentação diária respeita as porções na roda dos alimentos?" dataDxfId="23"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Quantas peças de fruta comes diariamente?" dataDxfId="22"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="E quantas porções (aproximadamente a palma da mão) de legumes comes diariamente?" dataDxfId="21"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Sabes o consumo calórico diário recomendado para ti?" dataDxfId="20"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Consultas algum nutricionista?" dataDxfId="19"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Relativamente à tua alimentação tens alguma restrição?" dataDxfId="18"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Quantas vezes consomes &quot;fast food&quot; mensalmente?" dataDxfId="17"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Praticas alguma atividade física fora da escola? (Excepto ginásio)" dataDxfId="16"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Qual atividade praticas?" dataDxfId="15"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="É uma atividade coletiva ou individual?" dataDxfId="14"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Quantas vezes praticas essa atividade semanalmente?" dataDxfId="13"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Frequentas o ginásio?" dataDxfId="12"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="Quantos dias por semana vais ao ginásio?" dataDxfId="11"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="Qual a duração média dos teus treinos? (ginásio)" dataDxfId="10"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="Tiveste alguma lesão grave associada ao desporto, nos últimos 2 anos? (ex: fraturas, roturas, etc...)" dataDxfId="9"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="No geral o teu exercício físico é..." dataDxfId="8"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="Quantas horas costumas dormir, por dia, em média, durante a semana?" dataDxfId="7"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="Quantas horas costumas dormir, por dia, em média, durante o fim de semana?" dataDxfId="6"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="Costumas assistir algum tipo de ecrã até 30min antes de te deitares?" dataDxfId="5"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="Costumas adormecer enquanto assistes conteúdos digital? (TV, Youtube, Netflix, TikTok, etc...)" dataDxfId="4"/>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0000-000022000000}" name="Costumas comer antes de te deitares?" dataDxfId="3"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Costumas praticar atividades intensivas perto da hora de dormir?" dataDxfId="2"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="Costumas tirar sestas durante o dia?" dataDxfId="1"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0000-000025000000}" name="Costumas deitar-te sempre por volta da mesma hora?" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -999,7 +967,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AK146"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1791,10 +1759,10 @@
         <v>42</v>
       </c>
       <c r="V8" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="W8" s="3" t="s">
         <v>66</v>
-      </c>
-      <c r="W8" s="3" t="s">
-        <v>67</v>
       </c>
       <c r="X8">
         <v>1</v>
@@ -1882,7 +1850,7 @@
         <v>2</v>
       </c>
       <c r="Q9" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R9" s="3" t="s">
         <v>63</v>
@@ -1948,10 +1916,10 @@
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G10" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>70</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>40</v>
@@ -1984,7 +1952,7 @@
         <v>44</v>
       </c>
       <c r="R10" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="S10" s="3" t="s">
         <v>46</v>
@@ -1996,10 +1964,10 @@
         <v>42</v>
       </c>
       <c r="V10" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="W10" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X10">
         <v>3</v>
@@ -2014,10 +1982,10 @@
         <v>48</v>
       </c>
       <c r="AB10" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="AC10" s="3" t="s">
         <v>73</v>
-      </c>
-      <c r="AC10" s="3" t="s">
-        <v>74</v>
       </c>
       <c r="AD10" s="3" t="s">
         <v>50</v>
@@ -2059,10 +2027,10 @@
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>40</v>
@@ -2119,7 +2087,7 @@
         <v>56</v>
       </c>
       <c r="AD11" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AE11" s="3" t="s">
         <v>51</v>
@@ -2158,10 +2126,10 @@
       </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>62</v>
@@ -2191,16 +2159,16 @@
         <v>2</v>
       </c>
       <c r="Q12" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R12" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="S12" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="T12" s="3" t="s">
         <v>78</v>
-      </c>
-      <c r="S12" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="T12" s="3" t="s">
-        <v>79</v>
       </c>
       <c r="U12" s="3" t="s">
         <v>46</v>
@@ -2257,10 +2225,10 @@
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>62</v>
@@ -2305,10 +2273,10 @@
         <v>42</v>
       </c>
       <c r="V13" s="3" t="s">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="W13" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X13">
         <v>2</v>
@@ -2363,13 +2331,13 @@
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="H14" s="3" t="s">
         <v>81</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>83</v>
       </c>
       <c r="I14" s="3">
         <v>164</v>
@@ -2462,10 +2430,10 @@
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>62</v>
@@ -2504,16 +2472,16 @@
         <v>46</v>
       </c>
       <c r="T15" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="U15" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="V15" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="W15" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="U15" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="V15" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="W15" s="3" t="s">
-        <v>86</v>
       </c>
       <c r="X15">
         <v>2</v>
@@ -2568,10 +2536,10 @@
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>62</v>
@@ -2604,7 +2572,7 @@
         <v>46</v>
       </c>
       <c r="R16" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="S16" s="3" t="s">
         <v>46</v>
@@ -2624,7 +2592,7 @@
         <v>3</v>
       </c>
       <c r="AA16" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="AB16" s="3" t="s">
         <v>46</v>
@@ -2672,10 +2640,10 @@
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>60</v>
@@ -2728,7 +2696,7 @@
         <v>4</v>
       </c>
       <c r="AA17" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="AB17" s="3" t="s">
         <v>46</v>
@@ -2832,7 +2800,7 @@
         <v>3</v>
       </c>
       <c r="AA18" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="AB18" s="3" t="s">
         <v>46</v>
@@ -2880,13 +2848,13 @@
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="H19" s="3" t="s">
         <v>81</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>83</v>
       </c>
       <c r="I19" s="2">
         <v>173</v>
@@ -2979,10 +2947,10 @@
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>40</v>
@@ -3078,13 +3046,13 @@
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I21" s="3">
         <v>181</v>
@@ -3126,10 +3094,10 @@
         <v>42</v>
       </c>
       <c r="V21" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="W21" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X21">
         <v>5</v>
@@ -3142,7 +3110,7 @@
         <v>42</v>
       </c>
       <c r="AC21" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AD21" s="3" t="s">
         <v>57</v>
@@ -3184,10 +3152,10 @@
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>62</v>
@@ -3226,7 +3194,7 @@
         <v>46</v>
       </c>
       <c r="T22" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U22" s="3" t="s">
         <v>46</v>
@@ -3241,7 +3209,7 @@
         <v>46</v>
       </c>
       <c r="AC22" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD22" s="3" t="s">
         <v>50</v>
@@ -3283,13 +3251,13 @@
       </c>
       <c r="E23" s="3"/>
       <c r="F23" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I23" s="3">
         <v>176</v>
@@ -3319,7 +3287,7 @@
         <v>44</v>
       </c>
       <c r="R23" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="S23" s="3" t="s">
         <v>46</v>
@@ -3387,10 +3355,10 @@
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>62</v>
@@ -3444,7 +3412,7 @@
         <v>42</v>
       </c>
       <c r="AC24" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD24" s="3" t="s">
         <v>50</v>
@@ -3486,13 +3454,13 @@
       </c>
       <c r="E25" s="3"/>
       <c r="F25" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="I25" s="2">
         <v>173</v>
@@ -3526,7 +3494,7 @@
         <v>46</v>
       </c>
       <c r="T25" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U25" s="3" t="s">
         <v>46</v>
@@ -3540,13 +3508,13 @@
         <v>3</v>
       </c>
       <c r="AA25" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="AB25" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="AC25" s="3" t="s">
         <v>87</v>
-      </c>
-      <c r="AB25" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="AC25" s="3" t="s">
-        <v>90</v>
       </c>
       <c r="AD25" s="3" t="s">
         <v>50</v>
@@ -3588,13 +3556,13 @@
       </c>
       <c r="E26" s="3"/>
       <c r="F26" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I26" s="2">
         <v>180</v>
@@ -3636,10 +3604,10 @@
         <v>42</v>
       </c>
       <c r="V26" s="3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="W26" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X26">
         <v>3</v>
@@ -3657,10 +3625,10 @@
         <v>46</v>
       </c>
       <c r="AC26" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="AD26" s="3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="AE26" s="3" t="s">
         <v>51</v>
@@ -3699,10 +3667,10 @@
       </c>
       <c r="E27" s="3"/>
       <c r="F27" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>60</v>
@@ -3761,7 +3729,7 @@
         <v>46</v>
       </c>
       <c r="AC27" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD27" s="3" t="s">
         <v>57</v>
@@ -3803,10 +3771,10 @@
       </c>
       <c r="E28" s="3"/>
       <c r="F28" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H28" s="3" t="s">
         <v>62</v>
@@ -3845,16 +3813,16 @@
         <v>46</v>
       </c>
       <c r="T28" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="U28" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="V28" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="W28" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="U28" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="V28" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="W28" s="3" t="s">
-        <v>86</v>
       </c>
       <c r="X28">
         <v>3</v>
@@ -3914,10 +3882,10 @@
       </c>
       <c r="E29" s="3"/>
       <c r="F29" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H29" s="3" t="s">
         <v>62</v>
@@ -3956,16 +3924,16 @@
         <v>46</v>
       </c>
       <c r="T29" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="U29" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="V29" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="W29" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="U29" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="V29" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="W29" s="3" t="s">
-        <v>86</v>
       </c>
       <c r="X29">
         <v>3</v>
@@ -3978,7 +3946,7 @@
         <v>42</v>
       </c>
       <c r="AC29" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AD29" s="3" t="s">
         <v>57</v>
@@ -4020,10 +3988,10 @@
       </c>
       <c r="E30" s="3"/>
       <c r="F30" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H30" s="3" t="s">
         <v>62</v>
@@ -4053,7 +4021,7 @@
         <v>2</v>
       </c>
       <c r="Q30" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R30" s="3" t="s">
         <v>45</v>
@@ -4062,7 +4030,7 @@
         <v>46</v>
       </c>
       <c r="T30" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U30" s="3" t="s">
         <v>46</v>
@@ -4077,7 +4045,7 @@
         <v>46</v>
       </c>
       <c r="AC30" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD30" s="3" t="s">
         <v>57</v>
@@ -4119,10 +4087,10 @@
       </c>
       <c r="E31" s="3"/>
       <c r="F31" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H31" s="3" t="s">
         <v>62</v>
@@ -4167,10 +4135,10 @@
         <v>42</v>
       </c>
       <c r="V31" s="3" t="s">
-        <v>100</v>
+        <v>121</v>
       </c>
       <c r="W31" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X31">
         <v>3</v>
@@ -4225,13 +4193,13 @@
       </c>
       <c r="E32" s="3"/>
       <c r="F32" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I32" s="2">
         <v>173</v>
@@ -4261,7 +4229,7 @@
         <v>44</v>
       </c>
       <c r="R32" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="S32" s="3" t="s">
         <v>46</v>
@@ -4273,10 +4241,10 @@
         <v>42</v>
       </c>
       <c r="V32" s="3" t="s">
-        <v>101</v>
+        <v>122</v>
       </c>
       <c r="W32" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X32">
         <v>5</v>
@@ -4294,7 +4262,7 @@
         <v>46</v>
       </c>
       <c r="AC32" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AD32" s="3" t="s">
         <v>57</v>
@@ -4336,13 +4304,13 @@
       </c>
       <c r="E33" s="3"/>
       <c r="F33" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I33" s="2">
         <v>170</v>
@@ -4392,13 +4360,13 @@
         <v>3</v>
       </c>
       <c r="AA33" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="AB33" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC33" s="3" t="s">
         <v>87</v>
-      </c>
-      <c r="AB33" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="AC33" s="3" t="s">
-        <v>90</v>
       </c>
       <c r="AD33" s="3" t="s">
         <v>57</v>
@@ -4440,13 +4408,13 @@
       </c>
       <c r="E34" s="3"/>
       <c r="F34" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G34" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="H34" s="3" t="s">
         <v>98</v>
-      </c>
-      <c r="H34" s="3" t="s">
-        <v>103</v>
       </c>
       <c r="I34" s="2">
         <v>185</v>
@@ -4471,7 +4439,7 @@
         <v>3</v>
       </c>
       <c r="Q34" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R34" s="3" t="s">
         <v>45</v>
@@ -4542,10 +4510,10 @@
       </c>
       <c r="E35" s="3"/>
       <c r="F35" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>60</v>
@@ -4578,7 +4546,7 @@
         <v>43</v>
       </c>
       <c r="R35" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="S35" s="3" t="s">
         <v>46</v>
@@ -4641,10 +4609,10 @@
       </c>
       <c r="E36" s="3"/>
       <c r="F36" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H36" s="3" t="s">
         <v>62</v>
@@ -4680,19 +4648,19 @@
         <v>45</v>
       </c>
       <c r="S36" s="3" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="T36" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U36" s="3" t="s">
         <v>42</v>
       </c>
       <c r="V36" s="3" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="W36" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X36">
         <v>1</v>
@@ -4747,10 +4715,10 @@
       </c>
       <c r="E37" s="3"/>
       <c r="F37" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H37" s="3" t="s">
         <v>62</v>
@@ -4807,7 +4775,7 @@
         <v>56</v>
       </c>
       <c r="AD37" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AE37" s="3" t="s">
         <v>58</v>
@@ -4846,10 +4814,10 @@
       </c>
       <c r="E38" s="3"/>
       <c r="F38" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H38" s="3" t="s">
         <v>62</v>
@@ -4894,10 +4862,10 @@
         <v>42</v>
       </c>
       <c r="V38" s="3" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="W38" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="X38">
         <v>3</v>
@@ -4909,7 +4877,7 @@
         <v>3</v>
       </c>
       <c r="AA38" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="AB38" s="3" t="s">
         <v>46</v>
@@ -4918,7 +4886,7 @@
         <v>49</v>
       </c>
       <c r="AD38" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AE38" s="3" t="s">
         <v>51</v>
@@ -4957,13 +4925,13 @@
       </c>
       <c r="E39" s="3"/>
       <c r="F39" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G39" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="G39" s="3" t="s">
-        <v>70</v>
-      </c>
       <c r="H39" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I39" s="2">
         <v>179</v>
@@ -4999,16 +4967,16 @@
         <v>46</v>
       </c>
       <c r="T39" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U39" s="3" t="s">
         <v>42</v>
       </c>
       <c r="V39" s="3" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="W39" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X39">
         <v>4</v>
@@ -5063,10 +5031,10 @@
       </c>
       <c r="E40" s="3"/>
       <c r="F40" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="H40" s="3" t="s">
         <v>60</v>
@@ -5162,10 +5130,10 @@
       </c>
       <c r="E41" s="3"/>
       <c r="F41" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="H41" s="3" t="s">
         <v>60</v>
@@ -5261,10 +5229,10 @@
       </c>
       <c r="E42" s="3"/>
       <c r="F42" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G42" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="G42" s="3" t="s">
-        <v>70</v>
       </c>
       <c r="H42" s="3" t="s">
         <v>40</v>
@@ -5301,16 +5269,16 @@
         <v>46</v>
       </c>
       <c r="T42" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U42" s="3" t="s">
         <v>42</v>
       </c>
       <c r="V42" s="3" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="W42" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X42">
         <v>2</v>
@@ -5323,7 +5291,7 @@
         <v>46</v>
       </c>
       <c r="AC42" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD42" s="3" t="s">
         <v>50</v>
@@ -5365,10 +5333,10 @@
       </c>
       <c r="E43" s="3"/>
       <c r="F43" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G43" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="G43" s="3" t="s">
-        <v>70</v>
       </c>
       <c r="H43" s="3" t="s">
         <v>40</v>
@@ -5427,7 +5395,7 @@
         <v>46</v>
       </c>
       <c r="AC43" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AD43" s="3" t="s">
         <v>57</v>
@@ -5469,10 +5437,10 @@
       </c>
       <c r="E44" s="3"/>
       <c r="F44" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="H44" s="3" t="s">
         <v>60</v>
@@ -5511,16 +5479,16 @@
         <v>46</v>
       </c>
       <c r="T44" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U44" s="3" t="s">
         <v>42</v>
       </c>
       <c r="V44" s="3" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="W44" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X44">
         <v>7</v>
@@ -5533,7 +5501,7 @@
         <v>42</v>
       </c>
       <c r="AC44" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="AD44" s="3" t="s">
         <v>57</v>
@@ -5575,10 +5543,10 @@
       </c>
       <c r="E45" s="3"/>
       <c r="F45" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="H45" s="3" t="s">
         <v>62</v>
@@ -5617,7 +5585,7 @@
         <v>46</v>
       </c>
       <c r="T45" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U45" s="3" t="s">
         <v>46</v>
@@ -5632,7 +5600,7 @@
         <v>46</v>
       </c>
       <c r="AC45" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD45" s="3" t="s">
         <v>57</v>
@@ -5674,13 +5642,13 @@
       </c>
       <c r="E46" s="3"/>
       <c r="F46" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="I46" s="2">
         <v>187</v>
@@ -5716,16 +5684,16 @@
         <v>46</v>
       </c>
       <c r="T46" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U46" s="3" t="s">
         <v>42</v>
       </c>
       <c r="V46" s="3" t="s">
-        <v>111</v>
+        <v>127</v>
       </c>
       <c r="W46" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X46">
         <v>4</v>
@@ -5780,10 +5748,10 @@
       </c>
       <c r="E47" s="3"/>
       <c r="F47" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="H47" s="3" t="s">
         <v>40</v>
@@ -5822,7 +5790,7 @@
         <v>46</v>
       </c>
       <c r="T47" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U47" s="3" t="s">
         <v>46</v>
@@ -5842,7 +5810,7 @@
         <v>46</v>
       </c>
       <c r="AC47" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD47" s="3" t="s">
         <v>51</v>
@@ -5884,13 +5852,13 @@
       </c>
       <c r="E48" s="3"/>
       <c r="F48" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I48" s="2">
         <v>185</v>
@@ -5920,7 +5888,7 @@
         <v>44</v>
       </c>
       <c r="R48" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="S48" s="3" t="s">
         <v>46</v>
@@ -5932,10 +5900,10 @@
         <v>42</v>
       </c>
       <c r="V48" s="3" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="W48" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="X48">
         <v>3</v>
@@ -5953,7 +5921,7 @@
         <v>46</v>
       </c>
       <c r="AC48" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AD48" s="3" t="s">
         <v>57</v>
@@ -5995,10 +5963,10 @@
       </c>
       <c r="E49" s="3"/>
       <c r="F49" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="H49" s="3" t="s">
         <v>62</v>
@@ -6035,16 +6003,16 @@
         <v>46</v>
       </c>
       <c r="T49" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="U49" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="V49" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="W49" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="U49" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="V49" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="W49" s="3" t="s">
-        <v>86</v>
       </c>
       <c r="X49">
         <v>1</v>
@@ -6057,10 +6025,10 @@
         <v>46</v>
       </c>
       <c r="AC49" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD49" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AE49" s="3" t="s">
         <v>57</v>
@@ -6099,10 +6067,10 @@
       </c>
       <c r="E50" s="3"/>
       <c r="F50" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G50" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="G50" s="3" t="s">
-        <v>70</v>
       </c>
       <c r="H50" s="3" t="s">
         <v>40</v>
@@ -6141,7 +6109,7 @@
         <v>46</v>
       </c>
       <c r="T50" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U50" s="3" t="s">
         <v>46</v>
@@ -6153,7 +6121,7 @@
       </c>
       <c r="AA50" s="3"/>
       <c r="AB50" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AC50" s="3" t="s">
         <v>49</v>
@@ -6198,7 +6166,7 @@
       </c>
       <c r="E51" s="3"/>
       <c r="F51" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G51" s="3" t="s">
         <v>61</v>
@@ -6240,7 +6208,7 @@
         <v>46</v>
       </c>
       <c r="T51" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U51" s="3" t="s">
         <v>46</v>
@@ -6255,7 +6223,7 @@
         <v>46</v>
       </c>
       <c r="AC51" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD51" s="3" t="s">
         <v>57</v>
@@ -6297,13 +6265,13 @@
       </c>
       <c r="E52" s="3"/>
       <c r="F52" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="I52" s="2">
         <v>181</v>
@@ -6330,7 +6298,7 @@
         <v>2</v>
       </c>
       <c r="Q52" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R52" s="3" t="s">
         <v>45</v>
@@ -6339,16 +6307,16 @@
         <v>46</v>
       </c>
       <c r="T52" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U52" s="3" t="s">
         <v>42</v>
       </c>
       <c r="V52" s="3" t="s">
-        <v>111</v>
+        <v>131</v>
       </c>
       <c r="W52" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X52">
         <v>4</v>
@@ -6358,7 +6326,7 @@
       </c>
       <c r="AA52" s="3"/>
       <c r="AB52" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AC52" s="3" t="s">
         <v>49</v>
@@ -6403,13 +6371,13 @@
       </c>
       <c r="E53" s="3"/>
       <c r="F53" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G53" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="G53" s="3" t="s">
-        <v>70</v>
-      </c>
       <c r="H53" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I53" s="2">
         <v>183</v>
@@ -6451,10 +6419,10 @@
         <v>42</v>
       </c>
       <c r="V53" s="3" t="s">
-        <v>114</v>
+        <v>83</v>
       </c>
       <c r="W53" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="X53">
         <v>1</v>
@@ -6509,10 +6477,10 @@
       </c>
       <c r="E54" s="3"/>
       <c r="F54" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H54" s="3" t="s">
         <v>40</v>
@@ -6551,7 +6519,7 @@
         <v>46</v>
       </c>
       <c r="T54" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U54" s="3" t="s">
         <v>46</v>
@@ -6571,7 +6539,7 @@
         <v>46</v>
       </c>
       <c r="AC54" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD54" s="3" t="s">
         <v>57</v>
@@ -6613,10 +6581,10 @@
       </c>
       <c r="E55" s="3"/>
       <c r="F55" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H55" s="3" t="s">
         <v>60</v>
@@ -6717,10 +6685,10 @@
       </c>
       <c r="E56" s="3"/>
       <c r="F56" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="H56" s="3" t="s">
         <v>40</v>
@@ -6750,25 +6718,25 @@
         <v>3</v>
       </c>
       <c r="Q56" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R56" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="S56" s="3" t="s">
         <v>46</v>
       </c>
       <c r="T56" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="U56" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="V56" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="W56" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="U56" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="V56" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="W56" s="3" t="s">
-        <v>86</v>
       </c>
       <c r="X56">
         <v>3</v>
@@ -6786,7 +6754,7 @@
         <v>46</v>
       </c>
       <c r="AC56" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AD56" s="3" t="s">
         <v>50</v>
@@ -6828,13 +6796,13 @@
       </c>
       <c r="E57" s="3"/>
       <c r="F57" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G57" s="3" t="s">
         <v>61</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I57" s="2">
         <v>175</v>
@@ -6927,13 +6895,13 @@
       </c>
       <c r="E58" s="3"/>
       <c r="F58" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I58" s="3">
         <v>169</v>
@@ -6967,7 +6935,7 @@
         <v>46</v>
       </c>
       <c r="T58" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U58" s="3" t="s">
         <v>46</v>
@@ -6982,10 +6950,10 @@
         <v>46</v>
       </c>
       <c r="AC58" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD58" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AE58" s="3" t="s">
         <v>58</v>
@@ -7024,13 +6992,13 @@
       </c>
       <c r="E59" s="3"/>
       <c r="F59" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I59" s="3">
         <v>160</v>
@@ -7080,7 +7048,7 @@
         <v>5</v>
       </c>
       <c r="AA59" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="AB59" s="3" t="s">
         <v>46</v>
@@ -7128,13 +7096,13 @@
       </c>
       <c r="E60" s="3"/>
       <c r="F60" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I60" s="2">
         <v>170</v>
@@ -7164,7 +7132,7 @@
         <v>44</v>
       </c>
       <c r="R60" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="S60" s="3" t="s">
         <v>46</v>
@@ -7184,13 +7152,13 @@
         <v>6</v>
       </c>
       <c r="AA60" s="3" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="AB60" s="3" t="s">
         <v>46</v>
       </c>
       <c r="AC60" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="AD60" s="3" t="s">
         <v>57</v>
@@ -7232,10 +7200,10 @@
       </c>
       <c r="E61" s="3"/>
       <c r="F61" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G61" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="G61" s="3" t="s">
-        <v>70</v>
       </c>
       <c r="H61" s="3" t="s">
         <v>40</v>
@@ -7280,10 +7248,10 @@
         <v>42</v>
       </c>
       <c r="V61" s="3" t="s">
-        <v>118</v>
+        <v>83</v>
       </c>
       <c r="W61" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X61">
         <v>1</v>
@@ -7296,7 +7264,7 @@
         <v>46</v>
       </c>
       <c r="AC61" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD61" s="3" t="s">
         <v>57</v>
@@ -7338,13 +7306,13 @@
       </c>
       <c r="E62" s="3"/>
       <c r="F62" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G62" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="G62" s="3" t="s">
-        <v>70</v>
-      </c>
       <c r="H62" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="I62" s="2">
         <v>185</v>
@@ -7380,16 +7348,16 @@
         <v>46</v>
       </c>
       <c r="T62" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U62" s="3" t="s">
         <v>42</v>
       </c>
       <c r="V62" s="3" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="W62" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X62">
         <v>1</v>
@@ -7548,13 +7516,13 @@
       </c>
       <c r="E64" s="3"/>
       <c r="F64" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="I64" s="2">
         <v>178</v>
@@ -7605,13 +7573,13 @@
         <v>46</v>
       </c>
       <c r="AC64" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD64" s="3" t="s">
         <v>57</v>
       </c>
       <c r="AE64" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AF64" s="3" t="s">
         <v>52</v>
@@ -7647,13 +7615,13 @@
       </c>
       <c r="E65" s="3"/>
       <c r="F65" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I65" s="2">
         <v>170</v>
@@ -7689,7 +7657,7 @@
         <v>46</v>
       </c>
       <c r="T65" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="U65" s="3" t="s">
         <v>46</v>
@@ -7703,7 +7671,7 @@
         <v>5</v>
       </c>
       <c r="AA65" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="AB65" s="3" t="s">
         <v>46</v>
@@ -7712,7 +7680,7 @@
         <v>49</v>
       </c>
       <c r="AD65" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AE65" s="3" t="s">
         <v>58</v>
@@ -7751,10 +7719,10 @@
       </c>
       <c r="E66" s="3"/>
       <c r="F66" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H66" s="3" t="s">
         <v>40</v>
@@ -7850,13 +7818,13 @@
       </c>
       <c r="E67" s="3"/>
       <c r="F67" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="H67" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="I67" s="3">
         <v>178</v>
@@ -7886,7 +7854,7 @@
         <v>44</v>
       </c>
       <c r="R67" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="S67" s="3" t="s">
         <v>46</v>
@@ -7898,10 +7866,10 @@
         <v>42</v>
       </c>
       <c r="V67" s="3" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="W67" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="X67">
         <v>5</v>
@@ -7922,7 +7890,7 @@
         <v>49</v>
       </c>
       <c r="AD67" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AE67" s="3" t="s">
         <v>57</v>
@@ -7961,13 +7929,13 @@
       </c>
       <c r="E68" s="3"/>
       <c r="F68" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I68" s="2">
         <v>180</v>
@@ -8009,10 +7977,10 @@
         <v>42</v>
       </c>
       <c r="V68" s="3" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="W68" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="X68">
         <v>3</v>
@@ -8031,7 +7999,7 @@
         <v>50</v>
       </c>
       <c r="AE68" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AF68" s="3" t="s">
         <v>42</v>
@@ -8070,7 +8038,7 @@
         <v>38</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="H69" s="3" t="s">
         <v>62</v>
@@ -8103,7 +8071,7 @@
         <v>43</v>
       </c>
       <c r="R69" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="S69" s="3" t="s">
         <v>46</v>
@@ -8124,7 +8092,7 @@
         <v>46</v>
       </c>
       <c r="AC69" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD69" s="3" t="s">
         <v>50</v>
@@ -8169,7 +8137,7 @@
         <v>38</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="H70" s="3" t="s">
         <v>62</v>
@@ -8206,7 +8174,7 @@
         <v>46</v>
       </c>
       <c r="T70" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U70" s="3" t="s">
         <v>46</v>
@@ -8269,7 +8237,7 @@
         <v>61</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I71" s="2">
         <v>170</v>
@@ -8309,10 +8277,10 @@
         <v>42</v>
       </c>
       <c r="V71" s="3" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="W71" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X71">
         <v>2</v>
@@ -8322,16 +8290,16 @@
       </c>
       <c r="AA71" s="3"/>
       <c r="AB71" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AC71" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD71" s="3" t="s">
         <v>50</v>
       </c>
       <c r="AE71" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AF71" s="3" t="s">
         <v>42</v>
@@ -8367,10 +8335,10 @@
       </c>
       <c r="E72" s="3"/>
       <c r="F72" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="H72" s="3" t="s">
         <v>62</v>
@@ -8413,10 +8381,10 @@
         <v>42</v>
       </c>
       <c r="V72" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="W72" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X72">
         <v>2</v>
@@ -8429,7 +8397,7 @@
         <v>46</v>
       </c>
       <c r="AC72" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD72" s="3" t="s">
         <v>57</v>
@@ -8471,13 +8439,13 @@
       </c>
       <c r="E73" s="3"/>
       <c r="F73" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="I73" s="2">
         <v>179</v>
@@ -8611,7 +8579,7 @@
         <v>43</v>
       </c>
       <c r="R74" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="S74" s="3" t="s">
         <v>46</v>
@@ -8637,7 +8605,7 @@
         <v>46</v>
       </c>
       <c r="AC74" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD74" s="3" t="s">
         <v>57</v>
@@ -8682,7 +8650,7 @@
         <v>38</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="H75" s="3" t="s">
         <v>60</v>
@@ -8721,16 +8689,16 @@
         <v>46</v>
       </c>
       <c r="T75" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U75" s="3" t="s">
         <v>42</v>
       </c>
       <c r="V75" s="3" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="W75" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X75">
         <v>1</v>
@@ -8743,7 +8711,7 @@
         <v>46</v>
       </c>
       <c r="AC75" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD75" s="3" t="s">
         <v>57</v>
@@ -8788,7 +8756,7 @@
         <v>38</v>
       </c>
       <c r="G76" s="3" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="H76" s="3" t="s">
         <v>62</v>
@@ -8827,7 +8795,7 @@
         <v>46</v>
       </c>
       <c r="T76" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U76" s="3" t="s">
         <v>46</v>
@@ -8892,10 +8860,10 @@
         <v>38</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I77" s="3">
         <v>158</v>
@@ -8931,7 +8899,7 @@
         <v>46</v>
       </c>
       <c r="T77" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U77" s="3" t="s">
         <v>46</v>
@@ -8946,7 +8914,7 @@
         <v>46</v>
       </c>
       <c r="AC77" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD77" s="3" t="s">
         <v>57</v>
@@ -8991,7 +8959,7 @@
         <v>38</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="H78" s="3" t="s">
         <v>62</v>
@@ -9090,10 +9058,10 @@
         <v>38</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="I79" s="3">
         <v>160</v>
@@ -9144,7 +9112,7 @@
         <v>46</v>
       </c>
       <c r="AC79" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD79" s="3" t="s">
         <v>51</v>
@@ -9189,10 +9157,10 @@
         <v>38</v>
       </c>
       <c r="G80" s="3" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I80" s="3">
         <v>159</v>
@@ -9243,13 +9211,13 @@
         <v>46</v>
       </c>
       <c r="AC80" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD80" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AE80" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AF80" s="3" t="s">
         <v>42</v>
@@ -9291,7 +9259,7 @@
         <v>61</v>
       </c>
       <c r="H81" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I81" s="2">
         <v>163</v>
@@ -9342,7 +9310,7 @@
         <v>46</v>
       </c>
       <c r="AC81" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD81" s="3" t="s">
         <v>57</v>
@@ -9387,7 +9355,7 @@
         <v>38</v>
       </c>
       <c r="G82" s="3" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="H82" s="3" t="s">
         <v>60</v>
@@ -9486,7 +9454,7 @@
         <v>38</v>
       </c>
       <c r="G83" s="3" t="s">
-        <v>128</v>
+        <v>111</v>
       </c>
       <c r="H83" s="3" t="s">
         <v>53</v>
@@ -9544,7 +9512,7 @@
         <v>50</v>
       </c>
       <c r="AE83" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AF83" s="3" t="s">
         <v>42</v>
@@ -9583,10 +9551,10 @@
         <v>38</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="H84" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I84" s="2">
         <v>179</v>
@@ -9622,16 +9590,16 @@
         <v>46</v>
       </c>
       <c r="T84" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U84" s="3" t="s">
         <v>42</v>
       </c>
       <c r="V84" s="3" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="W84" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X84">
         <v>7</v>
@@ -9644,7 +9612,7 @@
         <v>46</v>
       </c>
       <c r="AC84" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="AD84" s="3" t="s">
         <v>50</v>
@@ -9689,10 +9657,10 @@
         <v>38</v>
       </c>
       <c r="G85" s="3" t="s">
-        <v>128</v>
+        <v>111</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I85" s="2">
         <v>174</v>
@@ -9785,10 +9753,10 @@
       </c>
       <c r="E86" s="3"/>
       <c r="F86" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G86" s="3" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="H86" s="3" t="s">
         <v>60</v>
@@ -9833,10 +9801,10 @@
         <v>42</v>
       </c>
       <c r="V86" s="3" t="s">
-        <v>118</v>
+        <v>83</v>
       </c>
       <c r="W86" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="X86">
         <v>2</v>
@@ -9849,7 +9817,7 @@
         <v>46</v>
       </c>
       <c r="AC86" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD86" s="3" t="s">
         <v>50</v>
@@ -9927,7 +9895,7 @@
         <v>43</v>
       </c>
       <c r="R87" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="S87" s="3" t="s">
         <v>46</v>
@@ -9948,7 +9916,7 @@
         <v>46</v>
       </c>
       <c r="AC87" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD87" s="3" t="s">
         <v>50</v>
@@ -9993,10 +9961,10 @@
         <v>38</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I88" s="3">
         <v>162</v>
@@ -10047,7 +10015,7 @@
         <v>46</v>
       </c>
       <c r="AC88" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD88" s="3" t="s">
         <v>57</v>
@@ -10092,7 +10060,7 @@
         <v>38</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>131</v>
+        <v>113</v>
       </c>
       <c r="H89" s="3" t="s">
         <v>60</v>
@@ -10146,7 +10114,7 @@
         <v>46</v>
       </c>
       <c r="AC89" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD89" s="3" t="s">
         <v>57</v>
@@ -10188,10 +10156,10 @@
       </c>
       <c r="E90" s="3"/>
       <c r="F90" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G90" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H90" s="3" t="s">
         <v>62</v>
@@ -10245,7 +10213,7 @@
         <v>46</v>
       </c>
       <c r="AC90" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD90" s="3" t="s">
         <v>57</v>
@@ -10287,13 +10255,13 @@
       </c>
       <c r="E91" s="3"/>
       <c r="F91" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G91" s="3" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="H91" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I91" s="2">
         <v>169</v>
@@ -10342,7 +10310,7 @@
         <v>46</v>
       </c>
       <c r="AC91" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD91" s="3" t="s">
         <v>57</v>
@@ -10387,7 +10355,7 @@
         <v>38</v>
       </c>
       <c r="G92" s="3" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="H92" s="3" t="s">
         <v>60</v>
@@ -10447,7 +10415,7 @@
         <v>50</v>
       </c>
       <c r="AE92" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AF92" s="3" t="s">
         <v>42</v>
@@ -10483,10 +10451,10 @@
       </c>
       <c r="E93" s="3"/>
       <c r="F93" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G93" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H93" s="3" t="s">
         <v>60</v>
@@ -10516,7 +10484,7 @@
         <v>1</v>
       </c>
       <c r="Q93" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R93" s="3" t="s">
         <v>45</v>
@@ -10543,7 +10511,7 @@
         <v>56</v>
       </c>
       <c r="AD93" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AE93" s="3" t="s">
         <v>64</v>
@@ -10615,7 +10583,7 @@
         <v>1</v>
       </c>
       <c r="Q94" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R94" s="3" t="s">
         <v>45</v>
@@ -10650,7 +10618,7 @@
         <v>57</v>
       </c>
       <c r="AE94" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AF94" s="3" t="s">
         <v>42</v>
@@ -10722,7 +10690,7 @@
         <v>44</v>
       </c>
       <c r="R95" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="S95" s="3" t="s">
         <v>46</v>
@@ -10734,10 +10702,10 @@
         <v>42</v>
       </c>
       <c r="V95" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="W95" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X95">
         <v>4</v>
@@ -10755,7 +10723,7 @@
         <v>42</v>
       </c>
       <c r="AC95" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AD95" s="3" t="s">
         <v>57</v>
@@ -10800,10 +10768,10 @@
         <v>38</v>
       </c>
       <c r="G96" s="3" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="H96" s="3" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="I96" s="2">
         <v>165</v>
@@ -10830,10 +10798,10 @@
         <v>4</v>
       </c>
       <c r="Q96" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R96" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="S96" s="3" t="s">
         <v>46</v>
@@ -10853,13 +10821,13 @@
         <v>3</v>
       </c>
       <c r="AA96" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="AB96" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC96" s="3" t="s">
         <v>87</v>
-      </c>
-      <c r="AB96" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="AC96" s="3" t="s">
-        <v>90</v>
       </c>
       <c r="AD96" s="3" t="s">
         <v>57</v>
@@ -10901,10 +10869,10 @@
       </c>
       <c r="E97" s="3"/>
       <c r="F97" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G97" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H97" s="3" t="s">
         <v>62</v>
@@ -11000,10 +10968,10 @@
       </c>
       <c r="E98" s="3"/>
       <c r="F98" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G98" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="G98" s="3" t="s">
-        <v>70</v>
       </c>
       <c r="H98" s="3" t="s">
         <v>40</v>
@@ -11048,10 +11016,10 @@
         <v>42</v>
       </c>
       <c r="V98" s="3" t="s">
-        <v>134</v>
+        <v>115</v>
       </c>
       <c r="W98" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="X98">
         <v>4</v>
@@ -11069,7 +11037,7 @@
         <v>46</v>
       </c>
       <c r="AC98" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AD98" s="3" t="s">
         <v>57</v>
@@ -11111,13 +11079,13 @@
       </c>
       <c r="E99" s="3"/>
       <c r="F99" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G99" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H99" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I99" s="2">
         <v>185</v>
@@ -11153,16 +11121,16 @@
         <v>46</v>
       </c>
       <c r="T99" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U99" s="3" t="s">
         <v>42</v>
       </c>
       <c r="V99" s="3" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="W99" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X99">
         <v>4</v>
@@ -11223,7 +11191,7 @@
         <v>65</v>
       </c>
       <c r="H100" s="3" t="s">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="I100" s="2">
         <v>156</v>
@@ -11259,7 +11227,7 @@
         <v>46</v>
       </c>
       <c r="T100" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U100" s="3" t="s">
         <v>46</v>
@@ -11274,7 +11242,7 @@
         <v>46</v>
       </c>
       <c r="AC100" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD100" s="3" t="s">
         <v>57</v>
@@ -11316,10 +11284,10 @@
       </c>
       <c r="E101" s="3"/>
       <c r="F101" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G101" s="3" t="s">
-        <v>136</v>
+        <v>116</v>
       </c>
       <c r="H101" s="3" t="s">
         <v>62</v>
@@ -11349,7 +11317,7 @@
         <v>4</v>
       </c>
       <c r="Q101" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R101" s="3" t="s">
         <v>45</v>
@@ -11358,16 +11326,16 @@
         <v>46</v>
       </c>
       <c r="T101" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U101" s="3" t="s">
         <v>42</v>
       </c>
       <c r="V101" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="W101" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X101">
         <v>1</v>
@@ -11386,7 +11354,7 @@
         <v>50</v>
       </c>
       <c r="AE101" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AF101" s="3" t="s">
         <v>42</v>
@@ -11422,13 +11390,13 @@
       </c>
       <c r="E102" s="3"/>
       <c r="F102" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G102" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H102" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I102" s="2">
         <v>172</v>
@@ -11470,10 +11438,10 @@
         <v>42</v>
       </c>
       <c r="V102" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="W102" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="X102">
         <v>3</v>
@@ -11486,7 +11454,7 @@
         <v>46</v>
       </c>
       <c r="AC102" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD102" s="3" t="s">
         <v>57</v>
@@ -11528,13 +11496,13 @@
       </c>
       <c r="E103" s="3"/>
       <c r="F103" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G103" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H103" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I103" s="2">
         <v>171</v>
@@ -11576,10 +11544,10 @@
         <v>42</v>
       </c>
       <c r="V103" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="W103" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="X103">
         <v>3</v>
@@ -11592,7 +11560,7 @@
         <v>42</v>
       </c>
       <c r="AC103" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD103" s="3" t="s">
         <v>57</v>
@@ -11634,13 +11602,13 @@
       </c>
       <c r="E104" s="3"/>
       <c r="F104" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G104" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="G104" s="3" t="s">
-        <v>70</v>
-      </c>
       <c r="H104" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I104" s="2">
         <v>175</v>
@@ -11690,7 +11658,7 @@
         <v>3</v>
       </c>
       <c r="AA104" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="AB104" s="3" t="s">
         <v>46</v>
@@ -11699,7 +11667,7 @@
         <v>49</v>
       </c>
       <c r="AD104" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AE104" s="3" t="s">
         <v>51</v>
@@ -11738,13 +11706,13 @@
       </c>
       <c r="E105" s="3"/>
       <c r="F105" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G105" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H105" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I105" s="2">
         <v>175</v>
@@ -11796,7 +11764,7 @@
         <v>56</v>
       </c>
       <c r="AD105" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AE105" s="3" t="s">
         <v>51</v>
@@ -11835,10 +11803,10 @@
       </c>
       <c r="E106" s="3"/>
       <c r="F106" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G106" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H106" s="3" t="s">
         <v>40</v>
@@ -11871,7 +11839,7 @@
         <v>43</v>
       </c>
       <c r="R106" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="S106" s="3" t="s">
         <v>46</v>
@@ -11934,10 +11902,10 @@
       </c>
       <c r="E107" s="3"/>
       <c r="F107" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G107" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H107" s="3" t="s">
         <v>62</v>
@@ -11976,7 +11944,7 @@
         <v>46</v>
       </c>
       <c r="T107" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U107" s="3" t="s">
         <v>46</v>
@@ -12033,10 +12001,10 @@
       </c>
       <c r="E108" s="3"/>
       <c r="F108" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G108" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H108" s="3" t="s">
         <v>40</v>
@@ -12081,10 +12049,10 @@
         <v>42</v>
       </c>
       <c r="V108" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W108" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X108">
         <v>6</v>
@@ -12097,7 +12065,7 @@
         <v>46</v>
       </c>
       <c r="AC108" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="AD108" s="3" t="s">
         <v>51</v>
@@ -12145,7 +12113,7 @@
         <v>65</v>
       </c>
       <c r="H109" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I109" s="2">
         <v>168</v>
@@ -12181,16 +12149,16 @@
         <v>46</v>
       </c>
       <c r="T109" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U109" s="3" t="s">
         <v>42</v>
       </c>
       <c r="V109" s="3" t="s">
-        <v>139</v>
+        <v>117</v>
       </c>
       <c r="W109" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X109">
         <v>2</v>
@@ -12203,7 +12171,7 @@
         <v>46</v>
       </c>
       <c r="AC109" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD109" s="3" t="s">
         <v>50</v>
@@ -12245,13 +12213,13 @@
       </c>
       <c r="E110" s="3"/>
       <c r="F110" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G110" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H110" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I110" s="2">
         <v>175</v>
@@ -12287,7 +12255,7 @@
         <v>46</v>
       </c>
       <c r="T110" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U110" s="3" t="s">
         <v>46</v>
@@ -12302,7 +12270,7 @@
         <v>46</v>
       </c>
       <c r="AC110" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD110" s="3" t="s">
         <v>57</v>
@@ -12344,13 +12312,13 @@
       </c>
       <c r="E111" s="3"/>
       <c r="F111" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G111" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="H111" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I111" s="2">
         <v>170</v>
@@ -12386,16 +12354,16 @@
         <v>46</v>
       </c>
       <c r="T111" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U111" s="3" t="s">
         <v>42</v>
       </c>
       <c r="V111" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="W111" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X111">
         <v>2</v>
@@ -12408,7 +12376,7 @@
         <v>46</v>
       </c>
       <c r="AC111" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD111" s="3" t="s">
         <v>50</v>
@@ -12450,10 +12418,10 @@
       </c>
       <c r="E112" s="3"/>
       <c r="F112" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G112" s="3" t="s">
-        <v>136</v>
+        <v>116</v>
       </c>
       <c r="H112" s="3" t="s">
         <v>62</v>
@@ -12483,7 +12451,7 @@
         <v>4</v>
       </c>
       <c r="Q112" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R112" s="3" t="s">
         <v>63</v>
@@ -12498,10 +12466,10 @@
         <v>42</v>
       </c>
       <c r="V112" s="3" t="s">
-        <v>141</v>
+        <v>118</v>
       </c>
       <c r="W112" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X112">
         <v>2</v>
@@ -12514,7 +12482,7 @@
         <v>46</v>
       </c>
       <c r="AC112" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD112" s="3" t="s">
         <v>57</v>
@@ -12559,10 +12527,10 @@
         <v>38</v>
       </c>
       <c r="G113" s="3" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="H113" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I113" s="2">
         <v>170</v>
@@ -12598,7 +12566,7 @@
         <v>46</v>
       </c>
       <c r="T113" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="U113" s="3" t="s">
         <v>46</v>
@@ -12613,7 +12581,7 @@
         <v>46</v>
       </c>
       <c r="AC113" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD113" s="3" t="s">
         <v>57</v>
@@ -12658,10 +12626,10 @@
         <v>38</v>
       </c>
       <c r="G114" s="3" t="s">
-        <v>131</v>
+        <v>113</v>
       </c>
       <c r="H114" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I114" s="3">
         <v>160</v>
@@ -12697,7 +12665,7 @@
         <v>46</v>
       </c>
       <c r="T114" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="U114" s="3" t="s">
         <v>46</v>
@@ -12802,10 +12770,10 @@
         <v>42</v>
       </c>
       <c r="V115" s="3" t="s">
-        <v>118</v>
+        <v>83</v>
       </c>
       <c r="W115" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X115">
         <v>1</v>
@@ -12818,7 +12786,7 @@
         <v>46</v>
       </c>
       <c r="AC115" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD115" s="3" t="s">
         <v>57</v>
@@ -12866,7 +12834,7 @@
         <v>61</v>
       </c>
       <c r="H116" s="3" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="I116" s="3">
         <v>178</v>
@@ -12900,7 +12868,7 @@
         <v>46</v>
       </c>
       <c r="T116" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U116" s="3" t="s">
         <v>46</v>
@@ -12915,7 +12883,7 @@
         <v>42</v>
       </c>
       <c r="AC116" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD116" s="3" t="s">
         <v>57</v>
@@ -12957,10 +12925,10 @@
       </c>
       <c r="E117" s="3"/>
       <c r="F117" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G117" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H117" s="3" t="s">
         <v>62</v>
@@ -12990,10 +12958,10 @@
         <v>2</v>
       </c>
       <c r="Q117" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R117" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="S117" s="3" t="s">
         <v>46</v>
@@ -13061,10 +13029,10 @@
       </c>
       <c r="E118" s="3"/>
       <c r="F118" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G118" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="H118" s="3" t="s">
         <v>60</v>
@@ -13103,16 +13071,16 @@
         <v>46</v>
       </c>
       <c r="T118" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U118" s="3" t="s">
         <v>42</v>
       </c>
       <c r="V118" s="3" t="s">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="W118" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X118">
         <v>2</v>
@@ -13125,7 +13093,7 @@
         <v>46</v>
       </c>
       <c r="AC118" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD118" s="3" t="s">
         <v>57</v>
@@ -13167,10 +13135,10 @@
       </c>
       <c r="E119" s="3"/>
       <c r="F119" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G119" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="G119" s="3" t="s">
-        <v>70</v>
       </c>
       <c r="H119" s="3" t="s">
         <v>62</v>
@@ -13207,16 +13175,16 @@
         <v>46</v>
       </c>
       <c r="T119" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="U119" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="V119" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="W119" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="U119" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="V119" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="W119" s="3" t="s">
-        <v>86</v>
       </c>
       <c r="X119">
         <v>2</v>
@@ -13271,13 +13239,13 @@
       </c>
       <c r="E120" s="3"/>
       <c r="F120" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G120" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H120" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I120" s="2">
         <v>185</v>
@@ -13307,7 +13275,7 @@
         <v>44</v>
       </c>
       <c r="R120" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="S120" s="3" t="s">
         <v>46</v>
@@ -13319,10 +13287,10 @@
         <v>42</v>
       </c>
       <c r="V120" s="3" t="s">
-        <v>118</v>
+        <v>83</v>
       </c>
       <c r="W120" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="X120">
         <v>6</v>
@@ -13334,13 +13302,13 @@
         <v>5</v>
       </c>
       <c r="AA120" s="3" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="AB120" s="3" t="s">
         <v>46</v>
       </c>
       <c r="AC120" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="AD120" s="3" t="s">
         <v>57</v>
@@ -13382,10 +13350,10 @@
       </c>
       <c r="E121" s="3"/>
       <c r="F121" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G121" s="3" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="H121" s="3" t="s">
         <v>62</v>
@@ -13486,10 +13454,10 @@
       </c>
       <c r="E122" s="3"/>
       <c r="F122" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G122" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H122" s="3" t="s">
         <v>53</v>
@@ -13585,13 +13553,13 @@
       </c>
       <c r="E123" s="3"/>
       <c r="F123" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G123" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H123" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I123" s="2">
         <v>168</v>
@@ -13621,7 +13589,7 @@
         <v>44</v>
       </c>
       <c r="R123" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="S123" s="3" t="s">
         <v>46</v>
@@ -13647,7 +13615,7 @@
         <v>46</v>
       </c>
       <c r="AC123" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD123" s="3" t="s">
         <v>57</v>
@@ -13689,13 +13657,13 @@
       </c>
       <c r="E124" s="3"/>
       <c r="F124" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G124" s="3" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="H124" s="3" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="I124" s="2">
         <v>180</v>
@@ -13731,7 +13699,7 @@
         <v>46</v>
       </c>
       <c r="T124" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U124" s="3" t="s">
         <v>46</v>
@@ -13794,7 +13762,7 @@
         <v>61</v>
       </c>
       <c r="H125" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I125" s="2">
         <v>178</v>
@@ -13845,7 +13813,7 @@
         <v>46</v>
       </c>
       <c r="AC125" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD125" s="3" t="s">
         <v>57</v>
@@ -13935,10 +13903,10 @@
         <v>42</v>
       </c>
       <c r="V126" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="W126" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X126">
         <v>5</v>
@@ -13951,7 +13919,7 @@
         <v>42</v>
       </c>
       <c r="AC126" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AD126" s="3" t="s">
         <v>57</v>
@@ -13999,7 +13967,7 @@
         <v>61</v>
       </c>
       <c r="H127" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I127" s="3">
         <v>155</v>
@@ -14026,7 +13994,7 @@
         <v>4</v>
       </c>
       <c r="Q127" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R127" s="3" t="s">
         <v>45</v>
@@ -14041,10 +14009,10 @@
         <v>42</v>
       </c>
       <c r="V127" s="3" t="s">
-        <v>118</v>
+        <v>83</v>
       </c>
       <c r="W127" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X127">
         <v>2</v>
@@ -14057,7 +14025,7 @@
         <v>46</v>
       </c>
       <c r="AC127" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD127" s="3" t="s">
         <v>50</v>
@@ -14141,16 +14109,16 @@
         <v>46</v>
       </c>
       <c r="T128" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U128" s="3" t="s">
         <v>42</v>
       </c>
       <c r="V128" s="3" t="s">
-        <v>143</v>
+        <v>71</v>
       </c>
       <c r="W128" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X128">
         <v>3</v>
@@ -14163,7 +14131,7 @@
         <v>46</v>
       </c>
       <c r="AC128" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD128" s="3" t="s">
         <v>57</v>
@@ -14211,7 +14179,7 @@
         <v>59</v>
       </c>
       <c r="H129" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I129" s="3">
         <v>168</v>
@@ -14245,7 +14213,7 @@
         <v>46</v>
       </c>
       <c r="T129" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U129" s="3" t="s">
         <v>46</v>
@@ -14259,13 +14227,13 @@
         <v>3</v>
       </c>
       <c r="AA129" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="AB129" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC129" s="3" t="s">
         <v>87</v>
-      </c>
-      <c r="AB129" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="AC129" s="3" t="s">
-        <v>90</v>
       </c>
       <c r="AD129" s="3" t="s">
         <v>50</v>
@@ -14307,7 +14275,7 @@
       </c>
       <c r="E130" s="3"/>
       <c r="F130" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G130" s="3" t="s">
         <v>61</v>
@@ -14340,7 +14308,7 @@
         <v>5</v>
       </c>
       <c r="Q130" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R130" s="3" t="s">
         <v>63</v>
@@ -14349,7 +14317,7 @@
         <v>46</v>
       </c>
       <c r="T130" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U130" s="3" t="s">
         <v>46</v>
@@ -14364,7 +14332,7 @@
         <v>46</v>
       </c>
       <c r="AC130" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD130" s="3" t="s">
         <v>51</v>
@@ -14406,13 +14374,13 @@
       </c>
       <c r="E131" s="3"/>
       <c r="F131" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G131" s="3" t="s">
         <v>61</v>
       </c>
       <c r="H131" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I131" s="2">
         <v>163</v>
@@ -14442,7 +14410,7 @@
         <v>44</v>
       </c>
       <c r="R131" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="S131" s="3" t="s">
         <v>46</v>
@@ -14462,13 +14430,13 @@
         <v>6</v>
       </c>
       <c r="AA131" s="3" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="AB131" s="3" t="s">
         <v>46</v>
       </c>
       <c r="AC131" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AD131" s="3" t="s">
         <v>57</v>
@@ -14510,10 +14478,10 @@
       </c>
       <c r="E132" s="3"/>
       <c r="F132" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G132" s="3" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="H132" s="3" t="s">
         <v>40</v>
@@ -14552,16 +14520,16 @@
         <v>46</v>
       </c>
       <c r="T132" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U132" s="3" t="s">
         <v>42</v>
       </c>
       <c r="V132" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="W132" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X132">
         <v>1</v>
@@ -14616,13 +14584,13 @@
       </c>
       <c r="E133" s="3"/>
       <c r="F133" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G133" s="3" t="s">
         <v>61</v>
       </c>
       <c r="H133" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I133" s="2">
         <v>173</v>
@@ -14658,16 +14626,16 @@
         <v>46</v>
       </c>
       <c r="T133" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U133" s="3" t="s">
         <v>42</v>
       </c>
       <c r="V133" s="3" t="s">
-        <v>149</v>
+        <v>115</v>
       </c>
       <c r="W133" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X133">
         <v>2</v>
@@ -14685,7 +14653,7 @@
         <v>46</v>
       </c>
       <c r="AC133" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AD133" s="3" t="s">
         <v>51</v>
@@ -14727,7 +14695,7 @@
       </c>
       <c r="E134" s="3"/>
       <c r="F134" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G134" s="3" t="s">
         <v>61</v>
@@ -14769,16 +14737,16 @@
         <v>46</v>
       </c>
       <c r="T134" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U134" s="3" t="s">
         <v>42</v>
       </c>
       <c r="V134" s="5" t="s">
-        <v>144</v>
+        <v>118</v>
       </c>
       <c r="W134" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X134">
         <v>3</v>
@@ -14791,7 +14759,7 @@
         <v>42</v>
       </c>
       <c r="AC134" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD134" s="3" t="s">
         <v>50</v>
@@ -14833,13 +14801,13 @@
       </c>
       <c r="E135" s="3"/>
       <c r="F135" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G135" s="3" t="s">
         <v>61</v>
       </c>
       <c r="H135" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I135" s="2">
         <v>179</v>
@@ -14873,7 +14841,7 @@
         <v>46</v>
       </c>
       <c r="T135" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U135" s="3" t="s">
         <v>46</v>
@@ -14888,7 +14856,7 @@
         <v>46</v>
       </c>
       <c r="AC135" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD135" s="3" t="s">
         <v>57</v>
@@ -14930,7 +14898,7 @@
       </c>
       <c r="E136" s="3"/>
       <c r="F136" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G136" s="3" t="s">
         <v>61</v>
@@ -14987,7 +14955,7 @@
         <v>42</v>
       </c>
       <c r="AC136" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD136" s="3" t="s">
         <v>57</v>
@@ -15029,7 +14997,7 @@
       </c>
       <c r="E137" s="3"/>
       <c r="F137" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G137" s="3" t="s">
         <v>61</v>
@@ -15071,7 +15039,7 @@
         <v>46</v>
       </c>
       <c r="T137" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U137" s="3" t="s">
         <v>46</v>
@@ -15091,7 +15059,7 @@
         <v>46</v>
       </c>
       <c r="AC137" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD137" s="3" t="s">
         <v>57</v>
@@ -15133,7 +15101,7 @@
       </c>
       <c r="E138" s="3"/>
       <c r="F138" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G138" s="3" t="s">
         <v>61</v>
@@ -15175,7 +15143,7 @@
         <v>46</v>
       </c>
       <c r="T138" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U138" s="3" t="s">
         <v>46</v>
@@ -15190,7 +15158,7 @@
         <v>42</v>
       </c>
       <c r="AC138" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD138" s="3" t="s">
         <v>57</v>
@@ -15232,7 +15200,7 @@
       </c>
       <c r="E139" s="3"/>
       <c r="F139" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G139" s="3" t="s">
         <v>61</v>
@@ -15336,13 +15304,13 @@
       </c>
       <c r="E140" s="3"/>
       <c r="F140" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G140" s="3" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="H140" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I140" s="2">
         <v>175</v>
@@ -15378,7 +15346,7 @@
         <v>46</v>
       </c>
       <c r="T140" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U140" s="3" t="s">
         <v>46</v>
@@ -15392,7 +15360,7 @@
         <v>5</v>
       </c>
       <c r="AA140" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="AB140" s="3" t="s">
         <v>46</v>
@@ -15440,13 +15408,13 @@
       </c>
       <c r="E141" s="3"/>
       <c r="F141" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G141" s="3" t="s">
         <v>61</v>
       </c>
       <c r="H141" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I141" s="2">
         <v>175</v>
@@ -15473,7 +15441,7 @@
         <v>3</v>
       </c>
       <c r="Q141" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R141" s="3" t="s">
         <v>63</v>
@@ -15482,7 +15450,7 @@
         <v>46</v>
       </c>
       <c r="T141" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="U141" s="3" t="s">
         <v>46</v>
@@ -15496,13 +15464,13 @@
         <v>6</v>
       </c>
       <c r="AA141" s="3" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="AB141" s="3" t="s">
         <v>46</v>
       </c>
       <c r="AC141" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AD141" s="3" t="s">
         <v>57</v>
@@ -15544,7 +15512,7 @@
       </c>
       <c r="E142" s="3"/>
       <c r="F142" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G142" s="3" t="s">
         <v>61</v>
@@ -15580,26 +15548,19 @@
         <v>44</v>
       </c>
       <c r="R142" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="S142" s="3" t="s">
         <v>46</v>
       </c>
       <c r="T142" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="U142" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="V142" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="W142" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="X142">
-        <v>3</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="V142" s="3"/>
+      <c r="W142" s="3"/>
       <c r="Y142" s="3" t="s">
         <v>42</v>
       </c>
@@ -15619,7 +15580,7 @@
         <v>50</v>
       </c>
       <c r="AE142" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AF142" s="3" t="s">
         <v>46</v>
@@ -15655,10 +15616,10 @@
       </c>
       <c r="E143" s="3"/>
       <c r="F143" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G143" s="3" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="H143" s="3" t="s">
         <v>60</v>
@@ -15703,10 +15664,10 @@
         <v>42</v>
       </c>
       <c r="V143" s="3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="W143" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X143">
         <v>4</v>
@@ -15761,13 +15722,13 @@
       </c>
       <c r="E144" s="3"/>
       <c r="F144" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G144" s="3" t="s">
-        <v>146</v>
+        <v>119</v>
       </c>
       <c r="H144" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I144" s="3">
         <v>164</v>
@@ -15809,10 +15770,10 @@
         <v>42</v>
       </c>
       <c r="V144" s="3" t="s">
-        <v>147</v>
+        <v>120</v>
       </c>
       <c r="W144" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X144">
         <v>2</v>
@@ -15825,7 +15786,7 @@
         <v>42</v>
       </c>
       <c r="AC144" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD144" s="3" t="s">
         <v>50</v>
@@ -15867,13 +15828,13 @@
       </c>
       <c r="E145" s="3"/>
       <c r="F145" s="3" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G145" s="3" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="H145" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I145" s="2">
         <v>174</v>
@@ -15909,7 +15870,7 @@
         <v>46</v>
       </c>
       <c r="T145" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="U145" s="3" t="s">
         <v>46</v>
@@ -15924,7 +15885,7 @@
         <v>46</v>
       </c>
       <c r="AC145" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="AD145" s="3" t="s">
         <v>50</v>

</xml_diff>